<commit_message>
feat(F-NAR-016): TREE-DIF-006 fins distinctes, oral plus lié
Passe après apply : souvenirs de fin par chemin, moins de refrain.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-006.xlsx
+++ b/stories/arbres/TREE-DIF-006.xlsx
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une goutte quitte l'arrosoir. Elle fait ploc sur la dalle chaude. Derrière la maison, le jardin est minuscule. Ça sent la terre, et un peu la menthe. Un linge rose sèche près du cerisier. Les bottes de papa cuisent au soleil. Maman a laissé l'arrosoir dans les fleurs. En ce moment, Raphaël s'accroupit. Une petite tête penche, trop sèche. Elle a soif ! Je n'ai pas vu celle-là. Il reste des gouttes, tu crois ? Je les porte ! Il saisit l'arrosoir à deux mains. L'eau chante, puis elle danse. Doucement, elle n'aime pas les vagues. Je vais trop vite. Tu peux choisir une fleur. Une jaune attend près du bac. Une rouge attend près des tomates. Une bleue attend près du banc. Merci d'avoir vu sa soif. Quelle couleur, Raphaël ?</t>
+          <t>Une goutte quitte l'arrosoir. Elle fait ploc sur la dalle chaude. Derrière la maison, le jardin est minuscule. Ça sent la terre, et un peu la menthe. Un linge rose sèche près du cerisier. Les bottes de papa cuisent au soleil. Maman a laissé l'arrosoir dans les fleurs. En ce moment, Raphaël s'accroupit. Une petite tête penche, trop sèche. Elle a soif ! Je n'ai pas vu celle-là. Il reste des gouttes, tu crois ? Je les porte ! Il saisit l'arrosoir à deux mains. L'eau chante, puis elle danse. Doucement, elle n'aime pas les vagues. Je vais trop vite. Tu peux choisir une fleur. Une jaune attend près du bac. Plus loin, une rouge se tient près des tomates. À l'ombre, une bleue penche près du banc. Merci d'avoir vu sa soif. Quelle couleur, Raphaël ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une goutte quitte l'arrosoir. Elle fait ploc sur la dalle chaude. Derrière la maison, le jardin est minuscule. Ça sent la terre, et un peu la menthe. Un linge rose sèche près du cerisier. Les bottes de papa cuisent au soleil. Maman a laissé l'arrosoir dans les fleurs. En ce moment, Raphaël s'accroupit. Une petite tête penche, trop sèche. Elle a soif ! Je n'ai pas vu celle-là. Il reste des gouttes, tu crois ? Je les porte ! Il saisit l'arrosoir à deux mains. L'eau chante, puis elle danse. Doucement, elle n'aime pas les vagues. Je vais trop vite. Tu peux choisir une fleur. Une jaune attend près du bac. Une rouge attend près des tomates. Une bleue attend près du banc. Merci d'avoir vu sa soif. Quelle couleur, Raphaël ?</t>
+          <t>Une goutte quitte l'arrosoir. Elle fait ploc sur la dalle chaude. Derrière la maison, le jardin est minuscule. Ça sent la terre, et un peu la menthe. Un linge rose sèche près du cerisier. Les bottes de papa cuisent au soleil. Maman a laissé l'arrosoir dans les fleurs. En ce moment, Raphaël s'accroupit. Une petite tête penche, trop sèche. Elle a soif ! Je n'ai pas vu celle-là. Il reste des gouttes, tu crois ? Je les porte ! Il saisit l'arrosoir à deux mains. L'eau chante, puis elle danse. Doucement, elle n'aime pas les vagues. Je vais trop vite. Tu peux choisir une fleur. Une jaune attend près du bac. Plus loin, une rouge se tient près des tomates. À l'ombre, une bleue penche près du banc. Merci d'avoir vu sa soif. Quelle couleur, Raphaël ?</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1356,8 +1356,8 @@
 enfant-m|Je vais trop vite.
 maman|Tu peux choisir une fleur.
 narrateur|Une jaune attend près du bac.
-narrateur|Une rouge attend près des tomates.
-narrateur|Une bleue attend près du banc.
+narrateur|Plus loin, une rouge se tient près des tomates.
+narrateur|À l'ombre, une bleue penche près du banc.
 papa|Merci d'avoir vu sa soif.
 maman|Quelle couleur, Raphaël ?</t>
         </is>
@@ -2698,12 +2698,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet n'est plus qu'un murmure. Une abeille peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet fait à peine plic. Une abeille peut revenir.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet n'est plus qu'un murmure. Une abeille peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet fait à peine plic. Une abeille peut revenir.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2846,7 +2846,7 @@
 narrateur|La tête jaune se redresse un peu.
 narrateur|Raphaël gigote, puis il se tient.
 maman|Bravo, elle boit.
-narrateur|Le robinet n'est plus qu'un murmure.
+narrateur|Le robinet fait à peine plic.
 enfant-m|Une abeille peut revenir.</t>
         </is>
       </c>
@@ -2874,12 +2874,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. Un grain de sable sèche sur le pétale jaune.</t>
+          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Le bac garde un rond d'ombre. Un grain de sable sèche sur le pétale jaune.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. Un grain de sable sèche sur le pétale jaune.</t>
+          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Le bac garde un rond d'ombre. Un grain de sable sèche sur le pétale jaune.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -3018,8 +3018,7 @@
 narrateur|Ils restent près du bac, sans bouger beaucoup.
 maman|La marguerite a pris le temps.
 papa|Tes gouttes sont arrivées.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une abeille passe, puis s'en va.
+narrateur|Le bac garde un rond d'ombre.
 narrateur|Un grain de sable sèche sur le pétale jaune.</t>
         </is>
       </c>
@@ -3223,12 +3222,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. La tasse garde un rond de soleil.</t>
+          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. La petite tasse se tait. La tasse garde un rond de soleil.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. La tasse garde un rond de soleil.</t>
+          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. La petite tasse se tait. La tasse garde un rond de soleil.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3367,8 +3366,7 @@
 narrateur|La petite tasse repose près du bac.
 maman|Ta tasse a fait le voyage.
 papa|Tu as couru, l'eau non.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une abeille passe, puis s'en va.
+narrateur|La petite tasse se tait.
 narrateur|La tasse garde un rond de soleil.</t>
         </is>
       </c>
@@ -3572,12 +3570,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. L'ombre de papa reste un moment sur le bac.</t>
+          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Papa s'essuie les mains sur le linge rose. L'ombre de papa reste un moment sur le bac.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. L'ombre de papa reste un moment sur le bac.</t>
+          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Papa s'essuie les mains sur le linge rose. L'ombre de papa reste un moment sur le bac.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3716,8 +3714,7 @@
 narrateur|Papa repose l'arrosoir jaune près du bac.
 maman|Vous avez visé juste.
 papa|À deux, c'était plus calme.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une abeille passe, puis s'en va.
+narrateur|Papa s'essuie les mains sur le linge rose.
 narrateur|L'ombre de papa reste un moment sur le bac.</t>
         </is>
       </c>
@@ -4116,12 +4113,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau n'est plus qu'un murmure. Une abeille peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau fait à peine plic. Une abeille peut revenir.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau n'est plus qu'un murmure. Une abeille peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau fait à peine plic. Une abeille peut revenir.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4264,7 +4261,7 @@
 narrateur|La tête jaune se redresse un peu.
 narrateur|Raphaël gigote, puis il se tient.
 maman|Bravo, elle boit.
-narrateur|Le seau n'est plus qu'un murmure.
+narrateur|Le seau fait à peine plic.
 enfant-m|Une abeille peut revenir.</t>
         </is>
       </c>
@@ -4292,12 +4289,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. Le seau a un fond de sable, tout calme.</t>
+          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Le bac garde un rond d'ombre. Le seau a un fond de sable, tout calme.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. Le seau a un fond de sable, tout calme.</t>
+          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Le bac garde un rond d'ombre. Le seau a un fond de sable, tout calme.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4436,8 +4433,7 @@
 narrateur|Ils restent près du bac, sans bouger beaucoup.
 maman|La marguerite a pris le temps.
 papa|Tes gouttes sont arrivées.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une abeille passe, puis s'en va.
+narrateur|Le bac garde un rond d'ombre.
 narrateur|Le seau a un fond de sable, tout calme.</t>
         </is>
       </c>
@@ -4641,12 +4637,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. Une miette de sable brille dans la tasse.</t>
+          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. La petite tasse se tait. Une miette de sable brille dans la tasse.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. Une miette de sable brille dans la tasse.</t>
+          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. La petite tasse se tait. Une miette de sable brille dans la tasse.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4785,8 +4781,7 @@
 narrateur|La petite tasse repose près du bac.
 maman|Ta tasse a fait le voyage.
 papa|Tu as couru, l'eau non.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une abeille passe, puis s'en va.
+narrateur|La petite tasse se tait.
 narrateur|Une miette de sable brille dans la tasse.</t>
         </is>
       </c>
@@ -4990,12 +4985,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. Les orteils de Raphaël ont séché.</t>
+          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Papa s'essuie les mains sur le linge rose. Les orteils de Raphaël ont séché.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. Les orteils de Raphaël ont séché.</t>
+          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Papa s'essuie les mains sur le linge rose. Les orteils de Raphaël ont séché.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5134,8 +5129,7 @@
 narrateur|Papa repose l'arrosoir jaune près du bac.
 maman|Vous avez visé juste.
 papa|À deux, c'était plus calme.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une abeille passe, puis s'en va.
+narrateur|Papa s'essuie les mains sur le linge rose.
 narrateur|Les orteils de Raphaël ont séché.</t>
         </is>
       </c>
@@ -5534,12 +5528,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir n'est plus qu'un murmure. Une abeille peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir fait à peine plic. Une abeille peut revenir.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir n'est plus qu'un murmure. Une abeille peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du bac. Il penche l'arrosoir jaune, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête jaune se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir fait à peine plic. Une abeille peut revenir.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5682,7 +5676,7 @@
 narrateur|La tête jaune se redresse un peu.
 narrateur|Raphaël gigote, puis il se tient.
 maman|Bravo, elle boit.
-narrateur|L'arrosoir n'est plus qu'un murmure.
+narrateur|L'arrosoir fait à peine plic.
 enfant-m|Une abeille peut revenir.</t>
         </is>
       </c>
@@ -5710,12 +5704,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. L'abeille est revenue, tout près.</t>
+          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Le bac garde un rond d'ombre. L'abeille est revenue, tout près.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. L'abeille est revenue, tout près.</t>
+          <t>La tête jaune ne penche plus. Ils restent près du bac, sans bouger beaucoup. La marguerite a pris le temps. Tes gouttes sont arrivées. Le bac garde un rond d'ombre. L'abeille est revenue, tout près.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5854,8 +5848,7 @@
 narrateur|Ils restent près du bac, sans bouger beaucoup.
 maman|La marguerite a pris le temps.
 papa|Tes gouttes sont arrivées.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une abeille passe, puis s'en va.
+narrateur|Le bac garde un rond d'ombre.
 narrateur|L'abeille est revenue, tout près.</t>
         </is>
       </c>
@@ -6059,12 +6052,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. La dernière goutte de maman a voyagé.</t>
+          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. La petite tasse se tait. La dernière goutte de maman a voyagé.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. La dernière goutte de maman a voyagé.</t>
+          <t>La tête jaune ne penche plus. La petite tasse repose près du bac. Ta tasse a fait le voyage. Tu as couru, l'eau non. La petite tasse se tait. La dernière goutte de maman a voyagé.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -6203,8 +6196,7 @@
 narrateur|La petite tasse repose près du bac.
 maman|Ta tasse a fait le voyage.
 papa|Tu as couru, l'eau non.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une abeille passe, puis s'en va.
+narrateur|La petite tasse se tait.
 narrateur|La dernière goutte de maman a voyagé.</t>
         </is>
       </c>
@@ -6408,12 +6400,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. Le bec de l'arrosoir ne gicle plus.</t>
+          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Papa s'essuie les mains sur le linge rose. Le bec de l'arrosoir ne gicle plus.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une abeille passe, puis s'en va. Le bec de l'arrosoir ne gicle plus.</t>
+          <t>La tête jaune ne penche plus. Papa repose l'arrosoir jaune près du bac. Vous avez visé juste. À deux, c'était plus calme. Papa s'essuie les mains sur le linge rose. Le bec de l'arrosoir ne gicle plus.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6552,8 +6544,7 @@
 narrateur|Papa repose l'arrosoir jaune près du bac.
 maman|Vous avez visé juste.
 papa|À deux, c'était plus calme.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une abeille passe, puis s'en va.
+narrateur|Papa s'essuie les mains sur le linge rose.
 narrateur|Le bec de l'arrosoir ne gicle plus.</t>
         </is>
       </c>
@@ -7685,12 +7676,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet n'est plus qu'un murmure. Une coccinelle peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet fait à peine plic. Une coccinelle peut revenir.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet n'est plus qu'un murmure. Une coccinelle peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet fait à peine plic. Une coccinelle peut revenir.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7833,7 +7824,7 @@
 narrateur|La tête rouge se redresse un peu.
 narrateur|Raphaël gigote, puis il se tient.
 maman|Bravo, elle boit.
-narrateur|Le robinet n'est plus qu'un murmure.
+narrateur|Le robinet fait à peine plic.
 enfant-m|Une coccinelle peut revenir.</t>
         </is>
       </c>
@@ -7861,12 +7852,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. Une coccinelle s'est posée sur le bouton rouge.</t>
+          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Une tomate encore chaude brille à côté. Une coccinelle s'est posée sur le bouton rouge.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. Une coccinelle s'est posée sur le bouton rouge.</t>
+          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Une tomate encore chaude brille à côté. Une coccinelle s'est posée sur le bouton rouge.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -8005,8 +7996,7 @@
 narrateur|Ils restent près des tomates, sans bouger beaucoup.
 maman|Le coquelicot a pris le temps.
 papa|Tes gouttes sont arrivées.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une coccinelle passe, puis s'en va.
+narrateur|Une tomate encore chaude brille à côté.
 narrateur|Une coccinelle s'est posée sur le bouton rouge.</t>
         </is>
       </c>
@@ -8210,12 +8200,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. Une tomate a une goutte, pour de rire.</t>
+          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. La terre a un petit sourire mouillé. Une tomate a une goutte, pour de rire.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. Une tomate a une goutte, pour de rire.</t>
+          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. La terre a un petit sourire mouillé. Une tomate a une goutte, pour de rire.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -8354,8 +8344,7 @@
 narrateur|La petite tasse repose près des tomates.
 maman|Ta tasse a fait le voyage.
 papa|Tu as couru, l'eau non.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une coccinelle passe, puis s'en va.
+narrateur|La terre a un petit sourire mouillé.
 narrateur|Une tomate a une goutte, pour de rire.</t>
         </is>
       </c>
@@ -8559,12 +8548,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. Le filet du robinet s'est tu.</t>
+          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Les plants de tomates ne bougent plus. Le filet du robinet s'est tu.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. Le filet du robinet s'est tu.</t>
+          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Les plants de tomates ne bougent plus. Le filet du robinet s'est tu.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8703,8 +8692,7 @@
 narrateur|Papa repose l'arrosoir rouge près des tomates.
 maman|Vous avez visé juste.
 papa|À deux, c'était plus calme.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une coccinelle passe, puis s'en va.
+narrateur|Les plants de tomates ne bougent plus.
 narrateur|Le filet du robinet s'est tu.</t>
         </is>
       </c>
@@ -9102,12 +9090,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau n'est plus qu'un murmure. Une coccinelle peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau fait à peine plic. Une coccinelle peut revenir.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau n'est plus qu'un murmure. Une coccinelle peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau fait à peine plic. Une coccinelle peut revenir.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9250,7 +9238,7 @@
 narrateur|La tête rouge se redresse un peu.
 narrateur|Raphaël gigote, puis il se tient.
 maman|Bravo, elle boit.
-narrateur|Le seau n'est plus qu'un murmure.
+narrateur|Le seau fait à peine plic.
 enfant-m|Une coccinelle peut revenir.</t>
         </is>
       </c>
@@ -9278,12 +9266,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. La terre a cessé de faire des bulles.</t>
+          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Une tomate encore chaude brille à côté. La terre a cessé de faire des bulles.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. La terre a cessé de faire des bulles.</t>
+          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Une tomate encore chaude brille à côté. La terre a cessé de faire des bulles.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9422,8 +9410,7 @@
 narrateur|Ils restent près des tomates, sans bouger beaucoup.
 maman|Le coquelicot a pris le temps.
 papa|Tes gouttes sont arrivées.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une coccinelle passe, puis s'en va.
+narrateur|Une tomate encore chaude brille à côté.
 narrateur|La terre a cessé de faire des bulles.</t>
         </is>
       </c>
@@ -9627,12 +9614,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. La tasse a une auréole de terre.</t>
+          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. La terre a un petit sourire mouillé. La tasse a une auréole de terre.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. La tasse a une auréole de terre.</t>
+          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. La terre a un petit sourire mouillé. La tasse a une auréole de terre.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9771,8 +9758,7 @@
 narrateur|La petite tasse repose près des tomates.
 maman|Ta tasse a fait le voyage.
 papa|Tu as couru, l'eau non.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une coccinelle passe, puis s'en va.
+narrateur|La terre a un petit sourire mouillé.
 narrateur|La tasse a une auréole de terre.</t>
         </is>
       </c>
@@ -9976,12 +9962,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. Le seau repose entre les tomates.</t>
+          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Les plants de tomates ne bougent plus. Le seau repose entre les tomates.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. Le seau repose entre les tomates.</t>
+          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Les plants de tomates ne bougent plus. Le seau repose entre les tomates.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10120,8 +10106,7 @@
 narrateur|Papa repose l'arrosoir rouge près des tomates.
 maman|Vous avez visé juste.
 papa|À deux, c'était plus calme.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une coccinelle passe, puis s'en va.
+narrateur|Les plants de tomates ne bougent plus.
 narrateur|Le seau repose entre les tomates.</t>
         </is>
       </c>
@@ -10520,12 +10505,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir n'est plus qu'un murmure. Une coccinelle peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir fait à peine plic. Une coccinelle peut revenir.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir n'est plus qu'un murmure. Une coccinelle peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près des tomates. Il penche l'arrosoir rouge, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête rouge se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir fait à peine plic. Une coccinelle peut revenir.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -10668,7 +10653,7 @@
 narrateur|La tête rouge se redresse un peu.
 narrateur|Raphaël gigote, puis il se tient.
 maman|Bravo, elle boit.
-narrateur|L'arrosoir n'est plus qu'un murmure.
+narrateur|L'arrosoir fait à peine plic.
 enfant-m|Une coccinelle peut revenir.</t>
         </is>
       </c>
@@ -10696,12 +10681,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. Un pétale rouge a gardé une goutte ronde.</t>
+          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Une tomate encore chaude brille à côté. Un pétale rouge a gardé une goutte ronde.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. Un pétale rouge a gardé une goutte ronde.</t>
+          <t>La tête rouge ne penche plus. Ils restent près des tomates, sans bouger beaucoup. Le coquelicot a pris le temps. Tes gouttes sont arrivées. Une tomate encore chaude brille à côté. Un pétale rouge a gardé une goutte ronde.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -10840,8 +10825,7 @@
 narrateur|Ils restent près des tomates, sans bouger beaucoup.
 maman|Le coquelicot a pris le temps.
 papa|Tes gouttes sont arrivées.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une coccinelle passe, puis s'en va.
+narrateur|Une tomate encore chaude brille à côté.
 narrateur|Un pétale rouge a gardé une goutte ronde.</t>
         </is>
       </c>
@@ -11045,12 +11029,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. La coccinelle a repris le bec, tout doux.</t>
+          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. La terre a un petit sourire mouillé. La coccinelle a repris le bec, tout doux.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. La coccinelle a repris le bec, tout doux.</t>
+          <t>La tête rouge ne penche plus. La petite tasse repose près des tomates. Ta tasse a fait le voyage. Tu as couru, l'eau non. La terre a un petit sourire mouillé. La coccinelle a repris le bec, tout doux.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -11189,8 +11173,7 @@
 narrateur|La petite tasse repose près des tomates.
 maman|Ta tasse a fait le voyage.
 papa|Tu as couru, l'eau non.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une coccinelle passe, puis s'en va.
+narrateur|La terre a un petit sourire mouillé.
 narrateur|La coccinelle a repris le bec, tout doux.</t>
         </is>
       </c>
@@ -11394,12 +11377,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. L'arrosoir de maman s'est assis dans l'herbe.</t>
+          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Les plants de tomates ne bougent plus. L'arrosoir de maman s'est assis dans l'herbe.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Une coccinelle passe, puis s'en va. L'arrosoir de maman s'est assis dans l'herbe.</t>
+          <t>La tête rouge ne penche plus. Papa repose l'arrosoir rouge près des tomates. Vous avez visé juste. À deux, c'était plus calme. Les plants de tomates ne bougent plus. L'arrosoir de maman s'est assis dans l'herbe.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11538,8 +11521,7 @@
 narrateur|Papa repose l'arrosoir rouge près des tomates.
 maman|Vous avez visé juste.
 papa|À deux, c'était plus calme.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Une coccinelle passe, puis s'en va.
+narrateur|Les plants de tomates ne bougent plus.
 narrateur|L'arrosoir de maman s'est assis dans l'herbe.</t>
         </is>
       </c>
@@ -12671,12 +12653,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet n'est plus qu'un murmure. Un papillon peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet fait à peine plic. Un papillon peut revenir.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet n'est plus qu'un murmure. Un papillon peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le robinet fait à peine plic. Un papillon peut revenir.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12819,7 +12801,7 @@
 narrateur|La tête bleue se redresse un peu.
 narrateur|Raphaël gigote, puis il se tient.
 maman|Bravo, elle boit.
-narrateur|Le robinet n'est plus qu'un murmure.
+narrateur|Le robinet fait à peine plic.
 enfant-m|Un papillon peut revenir.</t>
         </is>
       </c>
@@ -12847,12 +12829,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Le zinc du robinet a une perle froide.</t>
+          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Une perle d'eau reste dans l'ombre. Le zinc du robinet a une perle froide.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Le zinc du robinet a une perle froide.</t>
+          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Une perle d'eau reste dans l'ombre. Le zinc du robinet a une perle froide.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -12991,8 +12973,7 @@
 narrateur|Ils restent près du banc, sans bouger beaucoup.
 maman|La fleur bleue a pris le temps.
 papa|Tes gouttes sont arrivées.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Un papillon passe, puis s'en va.
+narrateur|Une perle d'eau reste dans l'ombre.
 narrateur|Le zinc du robinet a une perle froide.</t>
         </is>
       </c>
@@ -13196,12 +13177,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Le bois du banc a un petit nuage mouillé.</t>
+          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Le bois sent encore la pluie d'hier. Le bois du banc a un petit nuage mouillé.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Le bois du banc a un petit nuage mouillé.</t>
+          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Le bois sent encore la pluie d'hier. Le bois du banc a un petit nuage mouillé.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13340,8 +13321,7 @@
 narrateur|La petite tasse repose près du banc.
 maman|Ta tasse a fait le voyage.
 papa|Tu as couru, l'eau non.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Un papillon passe, puis s'en va.
+narrateur|Le bois sent encore la pluie d'hier.
 narrateur|Le bois du banc a un petit nuage mouillé.</t>
         </is>
       </c>
@@ -13545,12 +13525,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Un papillon est resté sur l'anse bleue.</t>
+          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. L'ombre du banc a reculé d'un pas. Un papillon est resté sur l'anse bleue.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Un papillon est resté sur l'anse bleue.</t>
+          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. L'ombre du banc a reculé d'un pas. Un papillon est resté sur l'anse bleue.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -13689,8 +13669,7 @@
 narrateur|Papa repose l'arrosoir bleu près du banc.
 maman|Vous avez visé juste.
 papa|À deux, c'était plus calme.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Un papillon passe, puis s'en va.
+narrateur|L'ombre du banc a reculé d'un pas.
 narrateur|Un papillon est resté sur l'anse bleue.</t>
         </is>
       </c>
@@ -14089,12 +14068,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau n'est plus qu'un murmure. Un papillon peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau fait à peine plic. Un papillon peut revenir.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau n'est plus qu'un murmure. Un papillon peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. Le seau fait à peine plic. Un papillon peut revenir.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14237,7 +14216,7 @@
 narrateur|La tête bleue se redresse un peu.
 narrateur|Raphaël gigote, puis il se tient.
 maman|Bravo, elle boit.
-narrateur|Le seau n'est plus qu'un murmure.
+narrateur|Le seau fait à peine plic.
 enfant-m|Un papillon peut revenir.</t>
         </is>
       </c>
@@ -14265,12 +14244,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. L'ombre du seau a reculé, tout lent.</t>
+          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Une perle d'eau reste dans l'ombre. L'ombre du seau a reculé, tout lent.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. L'ombre du seau a reculé, tout lent.</t>
+          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Une perle d'eau reste dans l'ombre. L'ombre du seau a reculé, tout lent.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14409,8 +14388,7 @@
 narrateur|Ils restent près du banc, sans bouger beaucoup.
 maman|La fleur bleue a pris le temps.
 papa|Tes gouttes sont arrivées.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Un papillon passe, puis s'en va.
+narrateur|Une perle d'eau reste dans l'ombre.
 narrateur|L'ombre du seau a reculé, tout lent.</t>
         </is>
       </c>
@@ -14614,12 +14592,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. La tasse cliquette une dernière fois.</t>
+          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Le bois sent encore la pluie d'hier. La tasse cliquette une dernière fois.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. La tasse cliquette une dernière fois.</t>
+          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Le bois sent encore la pluie d'hier. La tasse cliquette une dernière fois.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14758,8 +14736,7 @@
 narrateur|La petite tasse repose près du banc.
 maman|Ta tasse a fait le voyage.
 papa|Tu as couru, l'eau non.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Un papillon passe, puis s'en va.
+narrateur|Le bois sent encore la pluie d'hier.
 narrateur|La tasse cliquette une dernière fois.</t>
         </is>
       </c>
@@ -14963,12 +14940,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Le seau d'ombre est rentré sous le banc.</t>
+          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. L'ombre du banc a reculé d'un pas. Le seau d'ombre est rentré sous le banc.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Le seau d'ombre est rentré sous le banc.</t>
+          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. L'ombre du banc a reculé d'un pas. Le seau d'ombre est rentré sous le banc.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15107,8 +15084,7 @@
 narrateur|Papa repose l'arrosoir bleu près du banc.
 maman|Vous avez visé juste.
 papa|À deux, c'était plus calme.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Un papillon passe, puis s'en va.
+narrateur|L'ombre du banc a reculé d'un pas.
 narrateur|Le seau d'ombre est rentré sous le banc.</t>
         </is>
       </c>
@@ -15507,12 +15483,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir n'est plus qu'un murmure. Un papillon peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir fait à peine plic. Un papillon peut revenir.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir n'est plus qu'un murmure. Un papillon peut revenir.</t>
+          <t>On attend les gouttes. Raphaël s'accroupit près du banc. Il penche l'arrosoir bleu, un tout petit peu. Une goutte tombe, puis une autre. Elle boit, tu vois ? La tête bleue se redresse un peu. Raphaël gigote, puis il se tient. Bravo, elle boit. L'arrosoir fait à peine plic. Un papillon peut revenir.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15655,7 +15631,7 @@
 narrateur|La tête bleue se redresse un peu.
 narrateur|Raphaël gigote, puis il se tient.
 maman|Bravo, elle boit.
-narrateur|L'arrosoir n'est plus qu'un murmure.
+narrateur|L'arrosoir fait à peine plic.
 enfant-m|Un papillon peut revenir.</t>
         </is>
       </c>
@@ -15683,12 +15659,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Une feuille d'ombre a bu, elle aussi.</t>
+          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Une perle d'eau reste dans l'ombre. Une feuille d'ombre a bu, elle aussi.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Une feuille d'ombre a bu, elle aussi.</t>
+          <t>La tête bleue ne penche plus. Ils restent près du banc, sans bouger beaucoup. La fleur bleue a pris le temps. Tes gouttes sont arrivées. Une perle d'eau reste dans l'ombre. Une feuille d'ombre a bu, elle aussi.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15827,8 +15803,7 @@
 narrateur|Ils restent près du banc, sans bouger beaucoup.
 maman|La fleur bleue a pris le temps.
 papa|Tes gouttes sont arrivées.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Un papillon passe, puis s'en va.
+narrateur|Une perle d'eau reste dans l'ombre.
 narrateur|Une feuille d'ombre a bu, elle aussi.</t>
         </is>
       </c>
@@ -16032,12 +16007,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Le papillon a suivi la tasse, puis parti.</t>
+          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Le bois sent encore la pluie d'hier. Le papillon a suivi la tasse, puis parti.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Le papillon a suivi la tasse, puis parti.</t>
+          <t>La tête bleue ne penche plus. La petite tasse repose près du banc. Ta tasse a fait le voyage. Tu as couru, l'eau non. Le bois sent encore la pluie d'hier. Le papillon a suivi la tasse, puis parti.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -16176,8 +16151,7 @@
 narrateur|La petite tasse repose près du banc.
 maman|Ta tasse a fait le voyage.
 papa|Tu as couru, l'eau non.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Un papillon passe, puis s'en va.
+narrateur|Le bois sent encore la pluie d'hier.
 narrateur|Le papillon a suivi la tasse, puis parti.</t>
         </is>
       </c>
@@ -16381,12 +16355,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Le bois du banc a séché, tout doux.</t>
+          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. L'ombre du banc a reculé d'un pas. Le bois du banc a séché, tout doux.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. Ça sent encore la menthe, tout près. Un papillon passe, puis s'en va. Le bois du banc a séché, tout doux.</t>
+          <t>La tête bleue ne penche plus. Papa repose l'arrosoir bleu près du banc. Vous avez visé juste. À deux, c'était plus calme. L'ombre du banc a reculé d'un pas. Le bois du banc a séché, tout doux.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16525,8 +16499,7 @@
 narrateur|Papa repose l'arrosoir bleu près du banc.
 maman|Vous avez visé juste.
 papa|À deux, c'était plus calme.
-narrateur|Ça sent encore la menthe, tout près.
-narrateur|Un papillon passe, puis s'en va.
+narrateur|L'ombre du banc a reculé d'un pas.
 narrateur|Le bois du banc a séché, tout doux.</t>
         </is>
       </c>
@@ -16548,7 +16521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16598,6 +16571,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>